<commit_message>
update info on calculations
</commit_message>
<xml_diff>
--- a/reductions/data/lit_dat.xlsx
+++ b/reductions/data/lit_dat.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="219" documentId="8_{7C4171F8-D199-4843-B714-C3F258BC4D93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D484913B-73F5-43B3-A6A4-9D9DF7B62CB7}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{DF353E34-80BC-440D-84E6-1A1BEACE8767}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{DF353E34-80BC-440D-84E6-1A1BEACE8767}"/>
   </bookViews>
   <sheets>
     <sheet name="Variable explanation" sheetId="2" r:id="rId1"/>
@@ -4458,14 +4458,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD7CE9C9-127E-4846-B34D-8BA0CB6E1A90}">
   <dimension ref="A1:C30"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.81640625" customWidth="1"/>
-    <col min="3" max="3" width="137.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" customWidth="1"/>
+    <col min="3" max="3" width="137.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4476,7 +4476,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -4487,7 +4487,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -4498,7 +4498,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -4509,7 +4509,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -4520,7 +4520,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>87</v>
       </c>
@@ -4531,7 +4531,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>88</v>
       </c>
@@ -4542,7 +4542,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -4553,7 +4553,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -4564,7 +4564,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -4575,7 +4575,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -4586,7 +4586,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -4597,7 +4597,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -4608,7 +4608,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -4619,7 +4619,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -4630,7 +4630,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>32</v>
       </c>
@@ -4641,7 +4641,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>55</v>
       </c>
@@ -4652,7 +4652,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>33</v>
       </c>
@@ -4663,7 +4663,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>7</v>
       </c>
@@ -4674,7 +4674,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>8</v>
       </c>
@@ -4685,7 +4685,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>9</v>
       </c>
@@ -4696,7 +4696,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>13</v>
       </c>
@@ -4707,7 +4707,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>62</v>
       </c>
@@ -4718,7 +4718,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>69</v>
       </c>
@@ -4729,7 +4729,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>72</v>
       </c>
@@ -4740,7 +4740,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>70</v>
       </c>
@@ -4751,7 +4751,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>71</v>
       </c>
@@ -4762,7 +4762,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>16</v>
       </c>
@@ -4773,7 +4773,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>79</v>
       </c>
@@ -4784,7 +4784,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>23</v>
       </c>
@@ -4806,53 +4806,53 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D35D03E-84A5-4E70-9EFA-07826CEBC622}">
   <dimension ref="A1:AY336"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.81640625" style="1"/>
-    <col min="2" max="2" width="14.1796875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="59.81640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="8.54296875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="9.81640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="6.453125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="22.453125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="21.54296875" style="2" customWidth="1"/>
-    <col min="9" max="10" width="19.453125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="8.85546875" style="1"/>
+    <col min="2" max="2" width="14.140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="59.85546875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="8.5703125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="6.42578125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="22.42578125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="21.5703125" style="2" customWidth="1"/>
+    <col min="9" max="10" width="19.42578125" style="2" customWidth="1"/>
     <col min="11" max="11" width="11" style="5" customWidth="1"/>
-    <col min="12" max="12" width="12.453125" style="5" customWidth="1"/>
+    <col min="12" max="12" width="12.42578125" style="5" customWidth="1"/>
     <col min="13" max="14" width="23" style="2" customWidth="1"/>
-    <col min="15" max="15" width="12.453125" style="2" customWidth="1"/>
-    <col min="16" max="16" width="15.54296875" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="8.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.1796875" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="21" width="11.1796875" style="1" customWidth="1"/>
-    <col min="22" max="22" width="7.54296875" style="1" customWidth="1"/>
-    <col min="23" max="23" width="9.1796875" style="2" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="10.54296875" style="2" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="10.54296875" style="2" customWidth="1"/>
-    <col min="27" max="28" width="9.453125" style="2" customWidth="1"/>
-    <col min="29" max="29" width="20.453125" style="2" customWidth="1"/>
-    <col min="30" max="31" width="44.54296875" style="1" customWidth="1"/>
-    <col min="32" max="33" width="18.453125" style="2" customWidth="1"/>
+    <col min="15" max="15" width="12.42578125" style="2" customWidth="1"/>
+    <col min="16" max="16" width="15.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="8.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="21" width="11.140625" style="1" customWidth="1"/>
+    <col min="22" max="22" width="7.5703125" style="1" customWidth="1"/>
+    <col min="23" max="23" width="9.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="10.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="10.5703125" style="2" customWidth="1"/>
+    <col min="27" max="28" width="9.42578125" style="2" customWidth="1"/>
+    <col min="29" max="29" width="20.42578125" style="2" customWidth="1"/>
+    <col min="30" max="31" width="44.5703125" style="1" customWidth="1"/>
+    <col min="32" max="33" width="18.42578125" style="2" customWidth="1"/>
     <col min="34" max="36" width="19" style="2" customWidth="1"/>
-    <col min="37" max="37" width="8.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="38" max="38" width="9" style="1" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="12.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="15" style="1" customWidth="1"/>
-    <col min="41" max="41" width="13.54296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="14.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="14.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="43" max="43" width="17" style="1" customWidth="1"/>
-    <col min="44" max="44" width="15.54296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="18.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="46" max="47" width="6.54296875" style="2" customWidth="1"/>
-    <col min="48" max="48" width="6.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="6.54296875" style="2" customWidth="1"/>
-    <col min="50" max="50" width="10.453125" style="1" customWidth="1"/>
-    <col min="51" max="51" width="27.54296875" style="1" customWidth="1"/>
-    <col min="52" max="52" width="11.54296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="53" max="16384" width="8.81640625" style="1"/>
+    <col min="44" max="44" width="15.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="46" max="47" width="6.5703125" style="2" customWidth="1"/>
+    <col min="48" max="48" width="6.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="6.5703125" style="2" customWidth="1"/>
+    <col min="50" max="50" width="10.42578125" style="1" customWidth="1"/>
+    <col min="51" max="51" width="27.5703125" style="1" customWidth="1"/>
+    <col min="52" max="52" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="53" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:51" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:51" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>974</v>
       </c>
@@ -5007,7 +5007,7 @@
         <v>980</v>
       </c>
     </row>
-    <row r="2" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -5155,7 +5155,7 @@
         <v>908</v>
       </c>
     </row>
-    <row r="3" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -5305,7 +5305,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="4" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>1</v>
       </c>
@@ -5449,7 +5449,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="5" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>1</v>
       </c>
@@ -5599,7 +5599,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="6" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>1</v>
       </c>
@@ -5741,7 +5741,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="7" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>1</v>
       </c>
@@ -5888,7 +5888,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="8" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>1</v>
       </c>
@@ -6030,7 +6030,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="9" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>1</v>
       </c>
@@ -6177,7 +6177,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="10" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>1</v>
       </c>
@@ -6319,7 +6319,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="11" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>1</v>
       </c>
@@ -6466,7 +6466,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="12" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>1</v>
       </c>
@@ -6608,7 +6608,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="13" spans="1:51" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:51" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="8">
         <v>1</v>
       </c>
@@ -6756,7 +6756,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="14" spans="1:51" s="8" customFormat="1" ht="27.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:51" s="8" customFormat="1" ht="27.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="8">
         <v>2</v>
       </c>
@@ -6901,7 +6901,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="15" spans="1:51" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:51" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>3</v>
       </c>
@@ -7039,7 +7039,7 @@
         <v>913</v>
       </c>
     </row>
-    <row r="16" spans="1:51" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:51" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="8">
         <v>3</v>
       </c>
@@ -7177,7 +7177,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="17" spans="1:51" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:51" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>5</v>
       </c>
@@ -7312,7 +7312,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="18" spans="1:51" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:51" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="8">
         <v>7</v>
       </c>
@@ -7451,7 +7451,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="19" spans="1:51" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:51" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>8</v>
       </c>
@@ -7590,7 +7590,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="20" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>8</v>
       </c>
@@ -7726,7 +7726,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="21" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>8</v>
       </c>
@@ -7865,7 +7865,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="22" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>8</v>
       </c>
@@ -8001,7 +8001,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="23" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>8</v>
       </c>
@@ -8137,7 +8137,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="24" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>8</v>
       </c>
@@ -8273,7 +8273,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="25" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>8</v>
       </c>
@@ -8408,7 +8408,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="26" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>8</v>
       </c>
@@ -8543,7 +8543,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="27" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>8</v>
       </c>
@@ -8679,7 +8679,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="28" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>8</v>
       </c>
@@ -8815,7 +8815,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="29" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>9</v>
       </c>
@@ -8955,7 +8955,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="30" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>9</v>
       </c>
@@ -9095,7 +9095,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="31" spans="1:51" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:51" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="8">
         <v>9</v>
       </c>
@@ -9236,7 +9236,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="32" spans="1:51" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:51" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>10</v>
       </c>
@@ -9373,7 +9373,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="33" spans="1:50" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:50" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="8">
         <v>10</v>
       </c>
@@ -9514,7 +9514,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="34" spans="1:50" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:50" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>14</v>
       </c>
@@ -9652,7 +9652,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="35" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>14</v>
       </c>
@@ -9790,7 +9790,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="36" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>14</v>
       </c>
@@ -9934,7 +9934,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="37" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>14</v>
       </c>
@@ -10078,7 +10078,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="38" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>14</v>
       </c>
@@ -10222,7 +10222,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="39" spans="1:50" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:50" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="8">
         <v>14</v>
       </c>
@@ -10368,7 +10368,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="40" spans="1:50" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:50" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>16</v>
       </c>
@@ -10510,7 +10510,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="41" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>16</v>
       </c>
@@ -10654,7 +10654,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="42" spans="1:50" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:50" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="8">
         <v>16</v>
       </c>
@@ -10799,7 +10799,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="43" spans="1:50" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:50" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>17</v>
       </c>
@@ -10881,7 +10881,7 @@
         <v>2.4390243902439024</v>
       </c>
     </row>
-    <row r="44" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>17</v>
       </c>
@@ -10963,7 +10963,7 @@
         <v>7.3170731707317076</v>
       </c>
     </row>
-    <row r="45" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>17</v>
       </c>
@@ -11045,7 +11045,7 @@
         <v>7.3170731707317076</v>
       </c>
     </row>
-    <row r="46" spans="1:50" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:50" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="8">
         <v>17</v>
       </c>
@@ -11135,7 +11135,7 @@
       </c>
       <c r="AW46" s="11"/>
     </row>
-    <row r="47" spans="1:50" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:50" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>18</v>
       </c>
@@ -11267,7 +11267,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="48" spans="1:50" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:50" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="8">
         <v>18</v>
       </c>
@@ -11404,7 +11404,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="49" spans="1:50" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:50" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>20</v>
       </c>
@@ -11546,7 +11546,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="50" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>20</v>
       </c>
@@ -11685,7 +11685,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="51" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>20</v>
       </c>
@@ -11824,7 +11824,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="52" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>20</v>
       </c>
@@ -11963,7 +11963,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="53" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>20</v>
       </c>
@@ -12102,7 +12102,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="54" spans="1:50" s="22" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:50" s="22" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>20</v>
       </c>
@@ -12244,7 +12244,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="55" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>20</v>
       </c>
@@ -12383,7 +12383,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="56" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>20</v>
       </c>
@@ -12522,7 +12522,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="57" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>20</v>
       </c>
@@ -12661,7 +12661,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="58" spans="1:50" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:50" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="8">
         <v>20</v>
       </c>
@@ -12801,7 +12801,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="59" spans="1:50" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:50" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>21</v>
       </c>
@@ -12945,7 +12945,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="60" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>21</v>
       </c>
@@ -13089,7 +13089,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="61" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>22</v>
       </c>
@@ -13226,7 +13226,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="62" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>22</v>
       </c>
@@ -13363,7 +13363,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="63" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>22</v>
       </c>
@@ -13498,7 +13498,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="64" spans="1:50" s="22" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:50" s="22" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>22</v>
       </c>
@@ -13636,7 +13636,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="65" spans="1:49" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:49" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>22</v>
       </c>
@@ -13771,7 +13771,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="66" spans="1:49" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:49" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>22</v>
       </c>
@@ -13906,7 +13906,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="67" spans="1:49" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:49" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>22</v>
       </c>
@@ -14041,7 +14041,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="68" spans="1:49" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:49" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>22</v>
       </c>
@@ -14176,7 +14176,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="69" spans="1:49" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:49" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <v>22</v>
       </c>
@@ -14311,7 +14311,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="70" spans="1:49" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:49" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="8">
         <v>22</v>
       </c>
@@ -14449,7 +14449,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="71" spans="1:49" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:49" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>23</v>
       </c>
@@ -14588,7 +14588,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="72" spans="1:49" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:49" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="8">
         <v>23</v>
       </c>
@@ -14730,7 +14730,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="73" spans="1:49" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:49" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <v>25</v>
       </c>
@@ -14873,7 +14873,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="74" spans="1:49" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:49" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>25</v>
       </c>
@@ -15016,7 +15016,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="75" spans="1:49" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:49" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="8">
         <v>25</v>
       </c>
@@ -15160,7 +15160,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="76" spans="1:49" s="8" customFormat="1" ht="27.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:49" s="8" customFormat="1" ht="27.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="8">
         <v>26</v>
       </c>
@@ -15297,7 +15297,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="77" spans="1:49" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:49" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>27</v>
       </c>
@@ -15434,7 +15434,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="78" spans="1:49" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:49" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
         <v>27</v>
       </c>
@@ -15571,7 +15571,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="79" spans="1:49" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:49" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
         <v>27</v>
       </c>
@@ -15708,7 +15708,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="80" spans="1:49" s="22" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:49" s="22" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="22">
         <v>27</v>
       </c>
@@ -15848,7 +15848,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="81" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
         <v>27</v>
       </c>
@@ -15985,7 +15985,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="82" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
         <v>27</v>
       </c>
@@ -16122,7 +16122,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="83" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
         <v>27</v>
       </c>
@@ -16259,7 +16259,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="84" spans="1:50" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:50" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A84" s="8">
         <v>27</v>
       </c>
@@ -16399,7 +16399,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="85" spans="1:50" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:50" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
         <v>28</v>
       </c>
@@ -16545,7 +16545,7 @@
         <v>8.3333333333333321</v>
       </c>
     </row>
-    <row r="86" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
         <v>28</v>
       </c>
@@ -16691,7 +16691,7 @@
         <v>58.63636363636364</v>
       </c>
     </row>
-    <row r="87" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
         <v>28</v>
       </c>
@@ -16837,7 +16837,7 @@
         <v>11.363636363636363</v>
       </c>
     </row>
-    <row r="88" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
         <v>28</v>
       </c>
@@ -16984,7 +16984,7 @@
         <v>36.679536679536682</v>
       </c>
     </row>
-    <row r="89" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
         <v>28</v>
       </c>
@@ -17131,7 +17131,7 @@
         <v>6.5512517125420446</v>
       </c>
     </row>
-    <row r="90" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
         <v>28</v>
       </c>
@@ -17277,7 +17277,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
         <v>28</v>
       </c>
@@ -17424,7 +17424,7 @@
         <v>34.234234234234236</v>
       </c>
     </row>
-    <row r="92" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
         <v>28</v>
       </c>
@@ -17571,7 +17571,7 @@
         <v>62.166891300749562</v>
       </c>
     </row>
-    <row r="93" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
         <v>28</v>
       </c>
@@ -17718,7 +17718,7 @@
         <v>9.9099099099099011</v>
       </c>
     </row>
-    <row r="94" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
         <v>28</v>
       </c>
@@ -17865,7 +17865,7 @@
         <v>23.273657289002564</v>
       </c>
     </row>
-    <row r="95" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
         <v>28</v>
       </c>
@@ -18012,7 +18012,7 @@
         <v>71.803069053708441</v>
       </c>
     </row>
-    <row r="96" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
         <v>28</v>
       </c>
@@ -18159,7 +18159,7 @@
         <v>42.455242966751925</v>
       </c>
     </row>
-    <row r="97" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
         <v>28</v>
       </c>
@@ -18306,7 +18306,7 @@
         <v>28.169014084507033</v>
       </c>
     </row>
-    <row r="98" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
         <v>28</v>
       </c>
@@ -18453,7 +18453,7 @@
         <v>64.967989756722162</v>
       </c>
     </row>
-    <row r="99" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
         <v>28</v>
       </c>
@@ -18600,7 +18600,7 @@
         <v>7.0422535211267583</v>
       </c>
     </row>
-    <row r="100" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
         <v>28</v>
       </c>
@@ -18747,7 +18747,7 @@
         <v>39.344262295081968</v>
       </c>
     </row>
-    <row r="101" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
         <v>28</v>
       </c>
@@ -18894,7 +18894,7 @@
         <v>60.000000000000007</v>
       </c>
     </row>
-    <row r="102" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="1">
         <v>28</v>
       </c>
@@ -19041,7 +19041,7 @@
         <v>60.655737704918032</v>
       </c>
     </row>
-    <row r="103" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="1">
         <v>28</v>
       </c>
@@ -19188,7 +19188,7 @@
         <v>30.705394190871377</v>
       </c>
     </row>
-    <row r="104" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="1">
         <v>28</v>
       </c>
@@ -19335,7 +19335,7 @@
         <v>48.091286307053934</v>
       </c>
     </row>
-    <row r="105" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="1">
         <v>28</v>
       </c>
@@ -19482,7 +19482,7 @@
         <v>32.780082987551864</v>
       </c>
     </row>
-    <row r="106" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="1">
         <v>28</v>
       </c>
@@ -19629,7 +19629,7 @@
         <v>-26.842105263157919</v>
       </c>
     </row>
-    <row r="107" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="1">
         <v>28</v>
       </c>
@@ -19776,7 +19776,7 @@
         <v>-7.1889952153110155</v>
       </c>
     </row>
-    <row r="108" spans="1:50" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="108" spans="1:50" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A108" s="8">
         <v>28</v>
       </c>
@@ -19925,7 +19925,7 @@
         <v>-46.842105263157904</v>
       </c>
     </row>
-    <row r="109" spans="1:50" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:50" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A109" s="1">
         <v>29</v>
       </c>
@@ -20070,7 +20070,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="110" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="1">
         <v>29</v>
       </c>
@@ -20215,7 +20215,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="111" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="1">
         <v>29</v>
       </c>
@@ -20360,7 +20360,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="112" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:50" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="1">
         <v>29</v>
       </c>
@@ -20505,7 +20505,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="113" spans="1:51" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="113" spans="1:51" s="8" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A113" s="8">
         <v>29</v>
       </c>
@@ -20651,7 +20651,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="114" spans="1:51" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:51" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A114" s="1">
         <v>31</v>
       </c>
@@ -20790,7 +20790,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="115" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="1">
         <v>31</v>
       </c>
@@ -20929,7 +20929,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="116" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="1">
         <v>31</v>
       </c>
@@ -21068,7 +21068,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="117" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:51" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="1">
         <v>31</v>
       </c>
@@ -21207,7 +21207,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="118" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="1">
         <v>31</v>
       </c>
@@ -21348,7 +21348,7 @@
       <c r="AX118" s="1"/>
       <c r="AY118" s="1"/>
     </row>
-    <row r="119" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="119" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A119" s="8">
         <v>31</v>
       </c>
@@ -21489,7 +21489,7 @@
       <c r="AX119" s="8"/>
       <c r="AY119" s="8"/>
     </row>
-    <row r="120" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A120" s="1">
         <v>32</v>
       </c>
@@ -21632,7 +21632,7 @@
       </c>
       <c r="AY120" s="1"/>
     </row>
-    <row r="121" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="1">
         <v>32</v>
       </c>
@@ -21775,7 +21775,7 @@
       </c>
       <c r="AY121" s="1"/>
     </row>
-    <row r="122" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="1">
         <v>32</v>
       </c>
@@ -21918,7 +21918,7 @@
       </c>
       <c r="AY122" s="1"/>
     </row>
-    <row r="123" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="1">
         <v>32</v>
       </c>
@@ -22061,7 +22061,7 @@
       </c>
       <c r="AY123" s="1"/>
     </row>
-    <row r="124" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="1">
         <v>32</v>
       </c>
@@ -22202,7 +22202,7 @@
       <c r="AX124" s="1"/>
       <c r="AY124" s="1"/>
     </row>
-    <row r="125" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="1">
         <v>32</v>
       </c>
@@ -22345,7 +22345,7 @@
       </c>
       <c r="AY125" s="1"/>
     </row>
-    <row r="126" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="1">
         <v>32</v>
       </c>
@@ -22488,7 +22488,7 @@
       </c>
       <c r="AY126" s="1"/>
     </row>
-    <row r="127" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="1">
         <v>32</v>
       </c>
@@ -22631,7 +22631,7 @@
       </c>
       <c r="AY127" s="1"/>
     </row>
-    <row r="128" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="1">
         <v>32</v>
       </c>
@@ -22772,7 +22772,7 @@
       <c r="AX128" s="1"/>
       <c r="AY128" s="1"/>
     </row>
-    <row r="129" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="1">
         <v>32</v>
       </c>
@@ -22913,7 +22913,7 @@
       <c r="AX129" s="1"/>
       <c r="AY129" s="1"/>
     </row>
-    <row r="130" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="1">
         <v>32</v>
       </c>
@@ -23054,7 +23054,7 @@
       <c r="AX130" s="1"/>
       <c r="AY130" s="36"/>
     </row>
-    <row r="131" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="1">
         <v>32</v>
       </c>
@@ -23195,7 +23195,7 @@
       <c r="AX131" s="1"/>
       <c r="AY131" s="36"/>
     </row>
-    <row r="132" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="132" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A132" s="8">
         <v>32</v>
       </c>
@@ -23336,7 +23336,7 @@
       <c r="AX132" s="8"/>
       <c r="AY132" s="36"/>
     </row>
-    <row r="133" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A133" s="1">
         <v>34</v>
       </c>
@@ -23485,7 +23485,7 @@
       <c r="AX133" s="1"/>
       <c r="AY133" s="3"/>
     </row>
-    <row r="134" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="1">
         <v>34</v>
       </c>
@@ -23634,7 +23634,7 @@
       <c r="AX134" s="1"/>
       <c r="AY134" s="1"/>
     </row>
-    <row r="135" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="1">
         <v>34</v>
       </c>
@@ -23784,7 +23784,7 @@
       <c r="AX135" s="1"/>
       <c r="AY135" s="1"/>
     </row>
-    <row r="136" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="1">
         <v>34</v>
       </c>
@@ -23934,7 +23934,7 @@
       <c r="AX136" s="1"/>
       <c r="AY136" s="1"/>
     </row>
-    <row r="137" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="1">
         <v>35</v>
       </c>
@@ -24075,7 +24075,7 @@
       <c r="AX137" s="1"/>
       <c r="AY137" s="1"/>
     </row>
-    <row r="138" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="1">
         <v>35</v>
       </c>
@@ -24216,7 +24216,7 @@
       <c r="AX138" s="1"/>
       <c r="AY138" s="1"/>
     </row>
-    <row r="139" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="1">
         <v>35</v>
       </c>
@@ -24357,7 +24357,7 @@
       <c r="AX139" s="1"/>
       <c r="AY139" s="1"/>
     </row>
-    <row r="140" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="1">
         <v>35</v>
       </c>
@@ -24498,7 +24498,7 @@
       <c r="AX140" s="1"/>
       <c r="AY140" s="1"/>
     </row>
-    <row r="141" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="1">
         <v>35</v>
       </c>
@@ -24639,7 +24639,7 @@
       <c r="AX141" s="1"/>
       <c r="AY141" s="1"/>
     </row>
-    <row r="142" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="1">
         <v>35</v>
       </c>
@@ -24780,7 +24780,7 @@
       <c r="AX142" s="1"/>
       <c r="AY142" s="1"/>
     </row>
-    <row r="143" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="1">
         <v>35</v>
       </c>
@@ -24921,7 +24921,7 @@
       <c r="AX143" s="1"/>
       <c r="AY143" s="1"/>
     </row>
-    <row r="144" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="144" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A144" s="8">
         <v>35</v>
       </c>
@@ -25062,7 +25062,7 @@
       <c r="AX144" s="8"/>
       <c r="AY144" s="8"/>
     </row>
-    <row r="145" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A145" s="1">
         <v>36</v>
       </c>
@@ -25203,7 +25203,7 @@
       <c r="AX145" s="36"/>
       <c r="AY145" s="1"/>
     </row>
-    <row r="146" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="1">
         <v>36</v>
       </c>
@@ -25344,7 +25344,7 @@
       <c r="AX146" s="36"/>
       <c r="AY146" s="1"/>
     </row>
-    <row r="147" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="1">
         <v>36</v>
       </c>
@@ -25485,7 +25485,7 @@
       <c r="AX147" s="36"/>
       <c r="AY147" s="1"/>
     </row>
-    <row r="148" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="1">
         <v>36</v>
       </c>
@@ -25626,7 +25626,7 @@
       <c r="AX148" s="36"/>
       <c r="AY148" s="1"/>
     </row>
-    <row r="149" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="1">
         <v>36</v>
       </c>
@@ -25767,7 +25767,7 @@
       <c r="AX149" s="36"/>
       <c r="AY149" s="1"/>
     </row>
-    <row r="150" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="1">
         <v>36</v>
       </c>
@@ -25908,7 +25908,7 @@
       <c r="AX150" s="36"/>
       <c r="AY150" s="1"/>
     </row>
-    <row r="151" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="1">
         <v>36</v>
       </c>
@@ -26049,7 +26049,7 @@
       <c r="AX151" s="36"/>
       <c r="AY151" s="1"/>
     </row>
-    <row r="152" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="1">
         <v>36</v>
       </c>
@@ -26190,7 +26190,7 @@
       <c r="AX152" s="36"/>
       <c r="AY152" s="1"/>
     </row>
-    <row r="153" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="1">
         <v>36</v>
       </c>
@@ -26331,7 +26331,7 @@
       <c r="AX153" s="36"/>
       <c r="AY153" s="1"/>
     </row>
-    <row r="154" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="1">
         <v>36</v>
       </c>
@@ -26472,7 +26472,7 @@
       <c r="AX154" s="36"/>
       <c r="AY154" s="1"/>
     </row>
-    <row r="155" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="1">
         <v>36</v>
       </c>
@@ -26613,7 +26613,7 @@
       <c r="AX155" s="36"/>
       <c r="AY155" s="1"/>
     </row>
-    <row r="156" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="1">
         <v>36</v>
       </c>
@@ -26754,7 +26754,7 @@
       <c r="AX156" s="36"/>
       <c r="AY156" s="1"/>
     </row>
-    <row r="157" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157" s="1">
         <v>36</v>
       </c>
@@ -26895,7 +26895,7 @@
       <c r="AX157" s="36"/>
       <c r="AY157" s="1"/>
     </row>
-    <row r="158" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A158" s="1">
         <v>36</v>
       </c>
@@ -27036,7 +27036,7 @@
       <c r="AX158" s="36"/>
       <c r="AY158" s="1"/>
     </row>
-    <row r="159" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="1">
         <v>36</v>
       </c>
@@ -27177,7 +27177,7 @@
       <c r="AX159" s="36"/>
       <c r="AY159" s="1"/>
     </row>
-    <row r="160" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="160" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A160" s="8">
         <v>36</v>
       </c>
@@ -27318,7 +27318,7 @@
       <c r="AX160" s="37"/>
       <c r="AY160" s="8"/>
     </row>
-    <row r="161" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A161" s="1">
         <v>37</v>
       </c>
@@ -27458,7 +27458,7 @@
       <c r="AX161" s="1"/>
       <c r="AY161" s="1"/>
     </row>
-    <row r="162" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A162" s="1">
         <v>38</v>
       </c>
@@ -27608,7 +27608,7 @@
       </c>
       <c r="AY162" s="1"/>
     </row>
-    <row r="163" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="1">
         <v>38</v>
       </c>
@@ -27756,7 +27756,7 @@
       <c r="AX163" s="1"/>
       <c r="AY163" s="1"/>
     </row>
-    <row r="164" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="1">
         <v>38</v>
       </c>
@@ -27904,7 +27904,7 @@
       <c r="AX164" s="1"/>
       <c r="AY164" s="1"/>
     </row>
-    <row r="165" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="165" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A165" s="8">
         <v>38</v>
       </c>
@@ -28052,7 +28052,7 @@
       <c r="AX165" s="8"/>
       <c r="AY165" s="8"/>
     </row>
-    <row r="166" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A166" s="1">
         <v>39</v>
       </c>
@@ -28195,7 +28195,7 @@
       </c>
       <c r="AY166" s="1"/>
     </row>
-    <row r="167" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A167" s="1">
         <v>39</v>
       </c>
@@ -28336,7 +28336,7 @@
       <c r="AX167" s="1"/>
       <c r="AY167" s="1"/>
     </row>
-    <row r="168" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="1">
         <v>39</v>
       </c>
@@ -28477,7 +28477,7 @@
       <c r="AX168" s="1"/>
       <c r="AY168" s="1"/>
     </row>
-    <row r="169" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A169" s="1">
         <v>39</v>
       </c>
@@ -28618,7 +28618,7 @@
       <c r="AX169" s="1"/>
       <c r="AY169" s="1"/>
     </row>
-    <row r="170" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="1">
         <v>39</v>
       </c>
@@ -28759,7 +28759,7 @@
       <c r="AX170" s="1"/>
       <c r="AY170" s="1"/>
     </row>
-    <row r="171" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="1">
         <v>39</v>
       </c>
@@ -28900,7 +28900,7 @@
       <c r="AX171" s="1"/>
       <c r="AY171" s="1"/>
     </row>
-    <row r="172" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A172" s="1">
         <v>39</v>
       </c>
@@ -29041,7 +29041,7 @@
       <c r="AX172" s="1"/>
       <c r="AY172" s="1"/>
     </row>
-    <row r="173" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="173" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A173" s="8">
         <v>39</v>
       </c>
@@ -29182,7 +29182,7 @@
       <c r="AX173" s="8"/>
       <c r="AY173" s="8"/>
     </row>
-    <row r="174" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="174" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A174" s="8">
         <v>40</v>
       </c>
@@ -29331,7 +29331,7 @@
       </c>
       <c r="AY174" s="8"/>
     </row>
-    <row r="175" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A175" s="1">
         <v>41</v>
       </c>
@@ -29468,7 +29468,7 @@
       </c>
       <c r="AY175" s="1"/>
     </row>
-    <row r="176" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" s="1">
         <v>41</v>
       </c>
@@ -29602,7 +29602,7 @@
       </c>
       <c r="AY176" s="1"/>
     </row>
-    <row r="177" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A177" s="1">
         <v>41</v>
       </c>
@@ -29737,7 +29737,7 @@
       <c r="AX177" s="1"/>
       <c r="AY177" s="1"/>
     </row>
-    <row r="178" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="1">
         <v>41</v>
       </c>
@@ -29872,7 +29872,7 @@
       <c r="AX178" s="1"/>
       <c r="AY178" s="1"/>
     </row>
-    <row r="179" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="1">
         <v>41</v>
       </c>
@@ -30007,7 +30007,7 @@
       <c r="AX179" s="1"/>
       <c r="AY179" s="1"/>
     </row>
-    <row r="180" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="1">
         <v>41</v>
       </c>
@@ -30142,7 +30142,7 @@
       <c r="AX180" s="1"/>
       <c r="AY180" s="1"/>
     </row>
-    <row r="181" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A181" s="1">
         <v>41</v>
       </c>
@@ -30277,7 +30277,7 @@
       <c r="AX181" s="1"/>
       <c r="AY181" s="1"/>
     </row>
-    <row r="182" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A182" s="1">
         <v>42</v>
       </c>
@@ -30424,7 +30424,7 @@
       </c>
       <c r="AY182" s="1"/>
     </row>
-    <row r="183" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="183" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A183" s="8">
         <v>42</v>
       </c>
@@ -30569,7 +30569,7 @@
       <c r="AX183" s="8"/>
       <c r="AY183" s="8"/>
     </row>
-    <row r="184" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A184" s="1">
         <v>43</v>
       </c>
@@ -30709,7 +30709,7 @@
       <c r="AX184" s="1"/>
       <c r="AY184" s="1"/>
     </row>
-    <row r="185" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A185" s="1">
         <v>43</v>
       </c>
@@ -30849,7 +30849,7 @@
       <c r="AX185" s="1"/>
       <c r="AY185" s="1"/>
     </row>
-    <row r="186" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A186" s="1">
         <v>43</v>
       </c>
@@ -30989,7 +30989,7 @@
       <c r="AX186" s="1"/>
       <c r="AY186" s="1"/>
     </row>
-    <row r="187" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A187" s="1">
         <v>44</v>
       </c>
@@ -31129,7 +31129,7 @@
       <c r="AX187" s="1"/>
       <c r="AY187" s="1"/>
     </row>
-    <row r="188" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A188" s="1">
         <v>44</v>
       </c>
@@ -31269,7 +31269,7 @@
       <c r="AX188" s="1"/>
       <c r="AY188" s="1"/>
     </row>
-    <row r="189" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A189" s="1">
         <v>44</v>
       </c>
@@ -31409,7 +31409,7 @@
       <c r="AX189" s="1"/>
       <c r="AY189" s="1"/>
     </row>
-    <row r="190" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A190" s="1">
         <v>44</v>
       </c>
@@ -31549,7 +31549,7 @@
       <c r="AX190" s="1"/>
       <c r="AY190" s="1"/>
     </row>
-    <row r="191" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A191" s="1">
         <v>44</v>
       </c>
@@ -31690,7 +31690,7 @@
       <c r="AX191" s="1"/>
       <c r="AY191" s="1"/>
     </row>
-    <row r="192" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A192" s="1">
         <v>44</v>
       </c>
@@ -31831,7 +31831,7 @@
       <c r="AX192" s="1"/>
       <c r="AY192" s="1"/>
     </row>
-    <row r="193" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A193" s="1">
         <v>44</v>
       </c>
@@ -31972,7 +31972,7 @@
       <c r="AX193" s="1"/>
       <c r="AY193" s="1"/>
     </row>
-    <row r="194" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A194" s="1">
         <v>45</v>
       </c>
@@ -32115,7 +32115,7 @@
       </c>
       <c r="AY194" s="1"/>
     </row>
-    <row r="195" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A195" s="1">
         <v>45</v>
       </c>
@@ -32256,7 +32256,7 @@
       <c r="AX195" s="1"/>
       <c r="AY195" s="1"/>
     </row>
-    <row r="196" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A196" s="1">
         <v>45</v>
       </c>
@@ -32397,7 +32397,7 @@
       <c r="AX196" s="1"/>
       <c r="AY196" s="1"/>
     </row>
-    <row r="197" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="1">
         <v>45</v>
       </c>
@@ -32538,7 +32538,7 @@
       <c r="AX197" s="1"/>
       <c r="AY197" s="1"/>
     </row>
-    <row r="198" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A198" s="1">
         <v>45</v>
       </c>
@@ -32679,7 +32679,7 @@
       <c r="AX198" s="1"/>
       <c r="AY198" s="1"/>
     </row>
-    <row r="199" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A199" s="1">
         <v>45</v>
       </c>
@@ -32820,7 +32820,7 @@
       <c r="AX199" s="1"/>
       <c r="AY199" s="1"/>
     </row>
-    <row r="200" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A200" s="1">
         <v>45</v>
       </c>
@@ -32961,7 +32961,7 @@
       <c r="AX200" s="1"/>
       <c r="AY200" s="1"/>
     </row>
-    <row r="201" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A201" s="1">
         <v>45</v>
       </c>
@@ -33102,7 +33102,7 @@
       <c r="AX201" s="1"/>
       <c r="AY201" s="1"/>
     </row>
-    <row r="202" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="202" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A202" s="1">
         <v>46</v>
       </c>
@@ -33248,7 +33248,7 @@
       </c>
       <c r="AY202" s="8"/>
     </row>
-    <row r="203" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A203" s="1">
         <v>46</v>
       </c>
@@ -33391,7 +33391,7 @@
       </c>
       <c r="AY203" s="1"/>
     </row>
-    <row r="204" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A204" s="1">
         <v>46</v>
       </c>
@@ -33532,7 +33532,7 @@
         <v>950</v>
       </c>
     </row>
-    <row r="205" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A205" s="1">
         <v>46</v>
       </c>
@@ -33671,7 +33671,7 @@
       <c r="AX205" s="1"/>
       <c r="AY205" s="3"/>
     </row>
-    <row r="206" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A206" s="1">
         <v>46</v>
       </c>
@@ -33810,7 +33810,7 @@
       <c r="AX206" s="1"/>
       <c r="AY206" s="3"/>
     </row>
-    <row r="207" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A207" s="1">
         <v>47</v>
       </c>
@@ -33951,7 +33951,7 @@
       <c r="AX207" s="1"/>
       <c r="AY207" s="1"/>
     </row>
-    <row r="208" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A208" s="1">
         <v>47</v>
       </c>
@@ -34092,7 +34092,7 @@
       <c r="AX208" s="1"/>
       <c r="AY208" s="1"/>
     </row>
-    <row r="209" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="209" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A209" s="8">
         <v>47</v>
       </c>
@@ -34233,7 +34233,7 @@
       <c r="AX209" s="8"/>
       <c r="AY209" s="8"/>
     </row>
-    <row r="210" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A210" s="1">
         <v>48</v>
       </c>
@@ -34382,7 +34382,7 @@
         <v>968</v>
       </c>
     </row>
-    <row r="211" spans="1:51" s="23" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:51" s="23" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A211" s="22">
         <v>48</v>
       </c>
@@ -34530,7 +34530,7 @@
       <c r="AX211" s="22"/>
       <c r="AY211" s="22"/>
     </row>
-    <row r="212" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A212" s="1">
         <v>48</v>
       </c>
@@ -34677,7 +34677,7 @@
       <c r="AX212" s="1"/>
       <c r="AY212" s="1"/>
     </row>
-    <row r="213" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="213" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A213" s="8">
         <v>48</v>
       </c>
@@ -34826,7 +34826,7 @@
       </c>
       <c r="AY213" s="8"/>
     </row>
-    <row r="214" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A214" s="1">
         <v>49</v>
       </c>
@@ -34975,7 +34975,7 @@
       <c r="AX214" s="1"/>
       <c r="AY214" s="1"/>
     </row>
-    <row r="215" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A215" s="1">
         <v>49</v>
       </c>
@@ -35124,7 +35124,7 @@
       <c r="AX215" s="1"/>
       <c r="AY215" s="1"/>
     </row>
-    <row r="216" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="216" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A216" s="8">
         <v>49</v>
       </c>
@@ -35273,7 +35273,7 @@
       <c r="AX216" s="8"/>
       <c r="AY216" s="8"/>
     </row>
-    <row r="217" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A217" s="1">
         <v>50</v>
       </c>
@@ -35416,7 +35416,7 @@
         <v>958</v>
       </c>
     </row>
-    <row r="218" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A218" s="1">
         <v>50</v>
       </c>
@@ -35557,7 +35557,7 @@
       <c r="AX218" s="1"/>
       <c r="AY218" s="1"/>
     </row>
-    <row r="219" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A219" s="1">
         <v>50</v>
       </c>
@@ -35698,7 +35698,7 @@
       <c r="AX219" s="1"/>
       <c r="AY219" s="1"/>
     </row>
-    <row r="220" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A220" s="1">
         <v>50</v>
       </c>
@@ -35840,7 +35840,7 @@
       <c r="AX220" s="1"/>
       <c r="AY220" s="1"/>
     </row>
-    <row r="221" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A221" s="1">
         <v>50</v>
       </c>
@@ -35982,7 +35982,7 @@
       <c r="AX221" s="1"/>
       <c r="AY221" s="1"/>
     </row>
-    <row r="222" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A222" s="1">
         <v>50</v>
       </c>
@@ -36124,7 +36124,7 @@
       <c r="AX222" s="1"/>
       <c r="AY222" s="1"/>
     </row>
-    <row r="223" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A223" s="1">
         <v>50</v>
       </c>
@@ -36266,7 +36266,7 @@
       <c r="AX223" s="1"/>
       <c r="AY223" s="1"/>
     </row>
-    <row r="224" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A224" s="1">
         <v>50</v>
       </c>
@@ -36408,7 +36408,7 @@
       <c r="AX224" s="1"/>
       <c r="AY224" s="1"/>
     </row>
-    <row r="225" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A225" s="1">
         <v>51</v>
       </c>
@@ -36556,7 +36556,7 @@
       </c>
       <c r="AY225" s="1"/>
     </row>
-    <row r="226" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A226" s="1">
         <v>51</v>
       </c>
@@ -36704,7 +36704,7 @@
       </c>
       <c r="AY226" s="1"/>
     </row>
-    <row r="227" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A227" s="1">
         <v>51</v>
       </c>
@@ -36852,7 +36852,7 @@
       </c>
       <c r="AY227" s="1"/>
     </row>
-    <row r="228" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A228" s="1">
         <v>51</v>
       </c>
@@ -37000,7 +37000,7 @@
       </c>
       <c r="AY228" s="1"/>
     </row>
-    <row r="229" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A229" s="1">
         <v>51</v>
       </c>
@@ -37148,7 +37148,7 @@
       </c>
       <c r="AY229" s="1"/>
     </row>
-    <row r="230" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A230" s="1">
         <v>51</v>
       </c>
@@ -37297,7 +37297,7 @@
       </c>
       <c r="AY230" s="1"/>
     </row>
-    <row r="231" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A231" s="1">
         <v>51</v>
       </c>
@@ -37447,7 +37447,7 @@
       </c>
       <c r="AY231" s="1"/>
     </row>
-    <row r="232" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A232" s="1">
         <v>51</v>
       </c>
@@ -37597,7 +37597,7 @@
       </c>
       <c r="AY232" s="1"/>
     </row>
-    <row r="233" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A233" s="1">
         <v>51</v>
       </c>
@@ -37747,7 +37747,7 @@
       </c>
       <c r="AY233" s="1"/>
     </row>
-    <row r="234" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A234" s="1">
         <v>51</v>
       </c>
@@ -37898,7 +37898,7 @@
       </c>
       <c r="AY234" s="1"/>
     </row>
-    <row r="235" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A235" s="1">
         <v>51</v>
       </c>
@@ -38049,7 +38049,7 @@
       </c>
       <c r="AY235" s="1"/>
     </row>
-    <row r="236" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A236" s="1">
         <v>51</v>
       </c>
@@ -38200,7 +38200,7 @@
       </c>
       <c r="AY236" s="1"/>
     </row>
-    <row r="237" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A237" s="1">
         <v>51</v>
       </c>
@@ -38349,7 +38349,7 @@
       </c>
       <c r="AY237" s="1"/>
     </row>
-    <row r="238" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A238" s="1">
         <v>51</v>
       </c>
@@ -38498,7 +38498,7 @@
       </c>
       <c r="AY238" s="1"/>
     </row>
-    <row r="239" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A239" s="1">
         <v>51</v>
       </c>
@@ -38647,7 +38647,7 @@
       </c>
       <c r="AY239" s="1"/>
     </row>
-    <row r="240" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A240" s="1">
         <v>51</v>
       </c>
@@ -38796,7 +38796,7 @@
       </c>
       <c r="AY240" s="1"/>
     </row>
-    <row r="241" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A241" s="1">
         <v>51</v>
       </c>
@@ -38945,7 +38945,7 @@
       </c>
       <c r="AY241" s="1"/>
     </row>
-    <row r="242" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A242" s="1">
         <v>51</v>
       </c>
@@ -39094,7 +39094,7 @@
       </c>
       <c r="AY242" s="1"/>
     </row>
-    <row r="243" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A243" s="1">
         <v>51</v>
       </c>
@@ -39243,7 +39243,7 @@
       </c>
       <c r="AY243" s="1"/>
     </row>
-    <row r="244" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A244" s="1">
         <v>51</v>
       </c>
@@ -39393,7 +39393,7 @@
       </c>
       <c r="AY244" s="1"/>
     </row>
-    <row r="245" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A245" s="1">
         <v>51</v>
       </c>
@@ -39543,7 +39543,7 @@
       </c>
       <c r="AY245" s="1"/>
     </row>
-    <row r="246" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A246" s="1">
         <v>51</v>
       </c>
@@ -39692,7 +39692,7 @@
       </c>
       <c r="AY246" s="1"/>
     </row>
-    <row r="247" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A247" s="1">
         <v>51</v>
       </c>
@@ -39842,7 +39842,7 @@
       </c>
       <c r="AY247" s="1"/>
     </row>
-    <row r="248" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A248" s="1">
         <v>51</v>
       </c>
@@ -39992,7 +39992,7 @@
       </c>
       <c r="AY248" s="1"/>
     </row>
-    <row r="249" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A249" s="1">
         <v>51</v>
       </c>
@@ -40140,7 +40140,7 @@
       </c>
       <c r="AY249" s="1"/>
     </row>
-    <row r="250" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A250" s="1">
         <v>51</v>
       </c>
@@ -40289,7 +40289,7 @@
       </c>
       <c r="AY250" s="1"/>
     </row>
-    <row r="251" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A251" s="1">
         <v>51</v>
       </c>
@@ -40437,7 +40437,7 @@
       </c>
       <c r="AY251" s="1"/>
     </row>
-    <row r="252" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A252" s="1">
         <v>51</v>
       </c>
@@ -40586,7 +40586,7 @@
       </c>
       <c r="AY252" s="1"/>
     </row>
-    <row r="253" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A253" s="1">
         <v>51</v>
       </c>
@@ -40735,7 +40735,7 @@
       </c>
       <c r="AY253" s="1"/>
     </row>
-    <row r="254" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A254" s="1">
         <v>51</v>
       </c>
@@ -40885,7 +40885,7 @@
       </c>
       <c r="AY254" s="1"/>
     </row>
-    <row r="255" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A255" s="1">
         <v>51</v>
       </c>
@@ -41034,7 +41034,7 @@
       </c>
       <c r="AY255" s="1"/>
     </row>
-    <row r="256" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A256" s="1">
         <v>51</v>
       </c>
@@ -41184,7 +41184,7 @@
       </c>
       <c r="AY256" s="1"/>
     </row>
-    <row r="257" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A257" s="1">
         <v>51</v>
       </c>
@@ -41334,7 +41334,7 @@
       </c>
       <c r="AY257" s="1"/>
     </row>
-    <row r="258" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A258" s="1">
         <v>51</v>
       </c>
@@ -41485,7 +41485,7 @@
       </c>
       <c r="AY258" s="1"/>
     </row>
-    <row r="259" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A259" s="1">
         <v>51</v>
       </c>
@@ -41635,7 +41635,7 @@
       </c>
       <c r="AY259" s="1"/>
     </row>
-    <row r="260" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A260" s="1">
         <v>51</v>
       </c>
@@ -41786,7 +41786,7 @@
       </c>
       <c r="AY260" s="1"/>
     </row>
-    <row r="261" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A261" s="1">
         <v>51</v>
       </c>
@@ -41937,7 +41937,7 @@
       </c>
       <c r="AY261" s="1"/>
     </row>
-    <row r="262" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A262" s="1">
         <v>51</v>
       </c>
@@ -42088,7 +42088,7 @@
       </c>
       <c r="AY262" s="1"/>
     </row>
-    <row r="263" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A263" s="1">
         <v>51</v>
       </c>
@@ -42239,7 +42239,7 @@
       </c>
       <c r="AY263" s="1"/>
     </row>
-    <row r="264" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A264" s="1">
         <v>51</v>
       </c>
@@ -42390,7 +42390,7 @@
       </c>
       <c r="AY264" s="1"/>
     </row>
-    <row r="265" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A265" s="1">
         <v>51</v>
       </c>
@@ -42541,7 +42541,7 @@
       </c>
       <c r="AY265" s="1"/>
     </row>
-    <row r="266" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A266" s="1">
         <v>51</v>
       </c>
@@ -42691,7 +42691,7 @@
       </c>
       <c r="AY266" s="1"/>
     </row>
-    <row r="267" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A267" s="1">
         <v>51</v>
       </c>
@@ -42841,7 +42841,7 @@
       </c>
       <c r="AY267" s="1"/>
     </row>
-    <row r="268" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A268" s="1">
         <v>51</v>
       </c>
@@ -42992,7 +42992,7 @@
       </c>
       <c r="AY268" s="1"/>
     </row>
-    <row r="269" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="269" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A269" s="8">
         <v>51</v>
       </c>
@@ -43143,7 +43143,7 @@
       </c>
       <c r="AY269" s="8"/>
     </row>
-    <row r="270" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A270" s="1">
         <v>55</v>
       </c>
@@ -43281,7 +43281,7 @@
       <c r="AX270" s="1"/>
       <c r="AY270" s="1"/>
     </row>
-    <row r="271" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="271" spans="1:51" s="11" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A271" s="8">
         <v>55</v>
       </c>
@@ -43419,7 +43419,7 @@
       <c r="AX271" s="8"/>
       <c r="AY271" s="8"/>
     </row>
-    <row r="272" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A272" s="1">
         <v>56</v>
       </c>
@@ -43564,7 +43564,7 @@
       <c r="AX272" s="1"/>
       <c r="AY272" s="1"/>
     </row>
-    <row r="273" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A273" s="1">
         <v>56</v>
       </c>
@@ -43708,7 +43708,7 @@
       <c r="AX273" s="1"/>
       <c r="AY273" s="1"/>
     </row>
-    <row r="274" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A274" s="1">
         <v>57</v>
       </c>
@@ -43813,7 +43813,7 @@
       <c r="AX274" s="1"/>
       <c r="AY274" s="1"/>
     </row>
-    <row r="275" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A275" s="1">
         <v>57</v>
       </c>
@@ -43918,7 +43918,7 @@
       <c r="AX275" s="1"/>
       <c r="AY275" s="1"/>
     </row>
-    <row r="276" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A276" s="1">
         <v>57</v>
       </c>
@@ -44023,7 +44023,7 @@
       <c r="AX276" s="1"/>
       <c r="AY276" s="1"/>
     </row>
-    <row r="277" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A277" s="1">
         <v>57</v>
       </c>
@@ -44123,7 +44123,7 @@
       <c r="AX277" s="1"/>
       <c r="AY277" s="1"/>
     </row>
-    <row r="278" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A278" s="1">
         <v>57</v>
       </c>
@@ -44223,7 +44223,7 @@
       <c r="AX278" s="1"/>
       <c r="AY278" s="1"/>
     </row>
-    <row r="279" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A279" s="1">
         <v>57</v>
       </c>
@@ -44323,7 +44323,7 @@
       <c r="AX279" s="1"/>
       <c r="AY279" s="1"/>
     </row>
-    <row r="280" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="280" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A280" s="1">
         <v>58</v>
       </c>
@@ -44429,7 +44429,7 @@
       <c r="AX280" s="1"/>
       <c r="AY280" s="1"/>
     </row>
-    <row r="281" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="281" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A281" s="1">
         <v>58</v>
       </c>
@@ -44536,7 +44536,7 @@
       <c r="AX281" s="1"/>
       <c r="AY281" s="1"/>
     </row>
-    <row r="282" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="282" spans="1:51" s="2" customFormat="1" ht="27.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A282" s="1">
         <v>58</v>
       </c>
@@ -44642,7 +44642,7 @@
       <c r="AX282" s="1"/>
       <c r="AY282" s="1"/>
     </row>
-    <row r="283" spans="1:51" ht="27.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="283" spans="1:51" ht="27.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A283" s="1">
         <v>58</v>
       </c>
@@ -44754,7 +44754,7 @@
       </c>
       <c r="AV283"/>
     </row>
-    <row r="284" spans="1:51" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="284" spans="1:51" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A284" s="1">
         <v>58</v>
       </c>
@@ -44864,7 +44864,7 @@
       </c>
       <c r="AV284"/>
     </row>
-    <row r="285" spans="1:51" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="285" spans="1:51" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A285" s="1">
         <v>58</v>
       </c>
@@ -44974,7 +44974,7 @@
       </c>
       <c r="AV285"/>
     </row>
-    <row r="286" spans="1:51" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="286" spans="1:51" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A286" s="1">
         <v>58</v>
       </c>
@@ -45084,7 +45084,7 @@
       </c>
       <c r="AV286"/>
     </row>
-    <row r="287" spans="1:51" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="287" spans="1:51" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A287" s="1">
         <v>58</v>
       </c>
@@ -45194,7 +45194,7 @@
       </c>
       <c r="AV287"/>
     </row>
-    <row r="288" spans="1:51" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="288" spans="1:51" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A288" s="1">
         <v>58</v>
       </c>
@@ -45303,7 +45303,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="289" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="289" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A289" s="1">
         <v>58</v>
       </c>
@@ -45412,7 +45412,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="290" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="290" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A290" s="1">
         <v>58</v>
       </c>
@@ -45521,7 +45521,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="291" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="291" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A291" s="1">
         <v>58</v>
       </c>
@@ -45630,7 +45630,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="292" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="292" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A292" s="1">
         <v>58</v>
       </c>
@@ -45739,7 +45739,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="293" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="293" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A293" s="1">
         <v>58</v>
       </c>
@@ -45848,7 +45848,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="294" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="294" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A294" s="1">
         <v>59</v>
       </c>
@@ -45929,7 +45929,7 @@
         <v>51.2</v>
       </c>
     </row>
-    <row r="295" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="295" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A295" s="1">
         <v>59</v>
       </c>
@@ -46010,7 +46010,7 @@
         <v>76.400000000000006</v>
       </c>
     </row>
-    <row r="296" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="296" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A296" s="1">
         <v>59</v>
       </c>
@@ -46091,7 +46091,7 @@
         <v>39.5</v>
       </c>
     </row>
-    <row r="297" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="297" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A297" s="1">
         <v>59</v>
       </c>
@@ -46172,7 +46172,7 @@
         <v>66.099999999999994</v>
       </c>
     </row>
-    <row r="298" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="298" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A298" s="1">
         <v>59</v>
       </c>
@@ -46253,7 +46253,7 @@
         <v>28.8</v>
       </c>
     </row>
-    <row r="299" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="299" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A299" s="1">
         <v>59</v>
       </c>
@@ -46334,7 +46334,7 @@
         <v>68.900000000000006</v>
       </c>
     </row>
-    <row r="300" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="300" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A300" s="1">
         <v>59</v>
       </c>
@@ -46415,7 +46415,7 @@
         <v>37.799999999999997</v>
       </c>
     </row>
-    <row r="301" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="301" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A301" s="1">
         <v>59</v>
       </c>
@@ -46496,7 +46496,7 @@
         <v>83.1</v>
       </c>
     </row>
-    <row r="302" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="302" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A302" s="1">
         <v>59</v>
       </c>
@@ -46577,7 +46577,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="303" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="303" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A303" s="1">
         <v>59</v>
       </c>
@@ -46658,7 +46658,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="304" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="304" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A304" s="1">
         <v>59</v>
       </c>
@@ -46739,7 +46739,7 @@
         <v>46.1</v>
       </c>
     </row>
-    <row r="305" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="305" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A305" s="1">
         <v>59</v>
       </c>
@@ -46820,7 +46820,7 @@
         <v>69.8</v>
       </c>
     </row>
-    <row r="306" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="306" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A306" s="1">
         <v>59</v>
       </c>
@@ -46901,7 +46901,7 @@
         <v>22.3</v>
       </c>
     </row>
-    <row r="307" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="307" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A307" s="1">
         <v>59</v>
       </c>
@@ -46982,7 +46982,7 @@
         <v>45.2</v>
       </c>
     </row>
-    <row r="308" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="308" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A308" s="1">
         <v>59</v>
       </c>
@@ -47063,7 +47063,7 @@
         <v>47.4</v>
       </c>
     </row>
-    <row r="309" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="309" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A309" s="1">
         <v>59</v>
       </c>
@@ -47144,7 +47144,7 @@
         <v>77.2</v>
       </c>
     </row>
-    <row r="310" spans="1:47" ht="73.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="310" spans="1:47" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A310" s="1">
         <v>60</v>
       </c>
@@ -47247,7 +47247,7 @@
         <v>67.34693877551021</v>
       </c>
     </row>
-    <row r="311" spans="1:47" ht="145.5" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:47" ht="150.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A311" s="1">
         <v>61</v>
       </c>
@@ -47358,7 +47358,7 @@
         <v>85.294117647058826</v>
       </c>
     </row>
-    <row r="312" spans="1:47" ht="145" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:47" ht="150" x14ac:dyDescent="0.25">
       <c r="A312" s="1">
         <v>61</v>
       </c>
@@ -47463,7 +47463,7 @@
         <v>20.588235294117649</v>
       </c>
     </row>
-    <row r="313" spans="1:47" ht="145" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:47" ht="150" x14ac:dyDescent="0.25">
       <c r="A313" s="1">
         <v>61</v>
       </c>
@@ -47574,7 +47574,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="314" spans="1:47" ht="145" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:47" ht="150" x14ac:dyDescent="0.25">
       <c r="A314" s="1">
         <v>61</v>
       </c>
@@ -47679,7 +47679,7 @@
         <v>30.76923076923077</v>
       </c>
     </row>
-    <row r="315" spans="1:47" ht="145" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:47" ht="150" x14ac:dyDescent="0.25">
       <c r="A315" s="1">
         <v>61</v>
       </c>
@@ -47790,7 +47790,7 @@
         <v>84.269662921348313</v>
       </c>
     </row>
-    <row r="316" spans="1:47" ht="145" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:47" ht="150" x14ac:dyDescent="0.25">
       <c r="A316" s="1">
         <v>61</v>
       </c>
@@ -47895,7 +47895,7 @@
         <v>10.1123595505618</v>
       </c>
     </row>
-    <row r="317" spans="1:47" ht="145" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:47" ht="150" x14ac:dyDescent="0.25">
       <c r="A317" s="1">
         <v>61</v>
       </c>
@@ -48004,7 +48004,7 @@
         <v>-11.034482758620699</v>
       </c>
     </row>
-    <row r="318" spans="1:47" ht="145" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:47" ht="150" x14ac:dyDescent="0.25">
       <c r="A318" s="1">
         <v>61</v>
       </c>
@@ -48113,7 +48113,7 @@
         <v>18.96551724137931</v>
       </c>
     </row>
-    <row r="319" spans="1:47" ht="145" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:47" ht="150" x14ac:dyDescent="0.25">
       <c r="A319" s="1">
         <v>61</v>
       </c>
@@ -48218,7 +48218,7 @@
         <v>2.631578947368427</v>
       </c>
     </row>
-    <row r="320" spans="1:47" ht="145" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:47" ht="150" x14ac:dyDescent="0.25">
       <c r="A320" s="1">
         <v>61</v>
       </c>
@@ -48323,7 +48323,7 @@
         <v>35.96491228070176</v>
       </c>
     </row>
-    <row r="321" spans="1:51" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:51" ht="75" x14ac:dyDescent="0.25">
       <c r="A321" s="1">
         <v>62</v>
       </c>
@@ -48358,7 +48358,7 @@
         <v>34.4</v>
       </c>
     </row>
-    <row r="322" spans="1:51" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:51" ht="75" x14ac:dyDescent="0.25">
       <c r="A322" s="1">
         <v>62</v>
       </c>
@@ -48393,7 +48393,7 @@
         <v>61.989795918367349</v>
       </c>
     </row>
-    <row r="323" spans="1:51" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:51" ht="75" x14ac:dyDescent="0.25">
       <c r="A323" s="1">
         <v>62</v>
       </c>
@@ -48428,7 +48428,7 @@
         <v>38.676844783715005</v>
       </c>
     </row>
-    <row r="324" spans="1:51" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:51" ht="75" x14ac:dyDescent="0.25">
       <c r="A324" s="1">
         <v>62</v>
       </c>
@@ -48463,7 +48463,7 @@
         <v>52.89473684210526</v>
       </c>
     </row>
-    <row r="325" spans="1:51" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:51" ht="75" x14ac:dyDescent="0.25">
       <c r="A325" s="1">
         <v>62</v>
       </c>
@@ -48498,7 +48498,7 @@
         <v>31.607629427792915</v>
       </c>
     </row>
-    <row r="326" spans="1:51" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:51" ht="75" x14ac:dyDescent="0.25">
       <c r="A326" s="1">
         <v>62</v>
       </c>
@@ -48533,7 +48533,7 @@
         <v>44.705882352941174</v>
       </c>
     </row>
-    <row r="327" spans="1:51" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:51" ht="75" x14ac:dyDescent="0.25">
       <c r="A327" s="1">
         <v>62</v>
       </c>
@@ -48568,7 +48568,7 @@
         <v>37.16577540106951</v>
       </c>
     </row>
-    <row r="328" spans="1:51" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:51" ht="75" x14ac:dyDescent="0.25">
       <c r="A328" s="1">
         <v>62</v>
       </c>
@@ -48603,7 +48603,7 @@
         <v>26.854219948849099</v>
       </c>
     </row>
-    <row r="329" spans="1:51" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:51" ht="75" x14ac:dyDescent="0.25">
       <c r="A329" s="1">
         <v>62</v>
       </c>
@@ -48638,7 +48638,7 @@
         <v>35.038363171355499</v>
       </c>
     </row>
-    <row r="330" spans="1:51" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:51" ht="75" x14ac:dyDescent="0.25">
       <c r="A330" s="1">
         <v>62</v>
       </c>
@@ -48673,7 +48673,7 @@
         <v>38.650306748466257</v>
       </c>
     </row>
-    <row r="331" spans="1:51" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:51" ht="75" x14ac:dyDescent="0.25">
       <c r="A331" s="1">
         <v>62</v>
       </c>
@@ -48708,7 +48708,7 @@
         <v>64.916467780429585</v>
       </c>
     </row>
-    <row r="332" spans="1:51" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:51" ht="75" x14ac:dyDescent="0.25">
       <c r="A332" s="1">
         <v>62</v>
       </c>
@@ -48743,7 +48743,7 @@
         <v>67.910447761194035</v>
       </c>
     </row>
-    <row r="333" spans="1:51" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:51" ht="90" x14ac:dyDescent="0.25">
       <c r="A333" s="1">
         <v>63</v>
       </c>
@@ -48775,7 +48775,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="334" spans="1:51" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:51" ht="90" x14ac:dyDescent="0.25">
       <c r="A334" s="1">
         <v>63</v>
       </c>
@@ -48801,7 +48801,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="335" spans="1:51" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:51" ht="90" x14ac:dyDescent="0.25">
       <c r="A335" s="1">
         <v>63</v>
       </c>
@@ -48827,7 +48827,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="336" spans="1:51" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:51" ht="90" x14ac:dyDescent="0.25">
       <c r="A336" s="1">
         <v>63</v>
       </c>

</xml_diff>